<commit_message>
chore: update Instagram report 2026-09-21 08:16
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/2026-09-21.xlsx
+++ b/instagram-daily-checker/reports/2026-09-21.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-21 07:44:32</t>
+          <t>取得日時：2026-09-21 08:16:46</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>365</t>
+          <t>366</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+3件</t>
+          <t>+4件</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-20T12:00:06+0000</t>
+          <t>2026-09-20T23:15:25+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">

</xml_diff>